<commit_message>
Add data validation, template sheets, and BoolDisplay API (#181)
</commit_message>
<xml_diff>
--- a/src/Excelsior.Tests/ColumnAttributeTests.Test.verified.xlsx
+++ b/src/Excelsior.Tests/ColumnAttributeTests.Test.verified.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="DeterministicId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="DeterministicId3"/>
   </sheets>
 </workbook>
 </file>
@@ -41,7 +41,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0"/>
     <xf fontId="1" fillId="0" borderId="0" applyFont="1" applyFill="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFont="0" applyFill="0" applyAlignment="1">
@@ -53,14 +53,24 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFont="0" applyFill="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFont="0" applyFill="0"/>
   </cellXfs>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
 </styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="1" max="1" width="15" style="5" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
@@ -128,5 +138,42 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:D3"/>
+  <conditionalFormatting sqref="A2:A3">
+    <cfRule type="containsBlanks" dxfId="0" priority="1">
+      <formula>LEN(TRIM(A2))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2:B3">
+    <cfRule type="containsBlanks" dxfId="0" priority="2">
+      <formula>LEN(TRIM(B2))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:D3">
+    <cfRule type="containsBlanks" dxfId="0" priority="3">
+      <formula>LEN(TRIM(D2))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="3">
+    <dataValidation type="custom" allowBlank="0" showErrorMessage="1" errorTitle="Invalid value" error="Must be a number." sqref="A2:A3">
+      <formula1>ISNUMBER(A2)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="0" showErrorMessage="1" errorTitle="Invalid value" error="This field is required." sqref="B2:B3">
+      <formula1>LEN(TRIM(B2))&gt;0</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="0" showErrorMessage="1" errorTitle="Invalid value" error="This field is required." sqref="D2:D3">
+      <formula1>LEN(TRIM(D2))&gt;0</formula1>
+    </dataValidation>
+  </dataValidations>
 </worksheet>
+</file>
+
+<file path=customXml/item.xml><?xml version="1.0" encoding="utf-8"?>
+<columnMetadata xmlns="https://github.com/SimonCropp/Excelsior/columnMetadata/v1">
+  <sheet name="Sheet1">
+    <column index="1" property="Id"/>
+    <column index="2" property="Name"/>
+    <column index="3" property="HireDate"/>
+    <column index="4" property="Email"/>
+  </sheet>
+</columnMetadata>
 </file>
</xml_diff>

<commit_message>
Fix default column widths (#206)
* Fix default column widths

* .

* .

* .

* Update Directory.Build.props
</commit_message>
<xml_diff>
--- a/src/Excelsior.Tests/ColumnAttributeTests.Test.verified.xlsx
+++ b/src/Excelsior.Tests/ColumnAttributeTests.Test.verified.xlsx
@@ -70,9 +70,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col min="1" max="1" width="15" style="5" customWidth="1"/>
+    <col min="1" max="1" width="16" style="5" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="13" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>